<commit_message>
feat: Hot Deal is now called Offers
Same category, same handle (/categories/hot-deals still works), renamed
in the admin to match what it now holds: exactly the flowers with a
government-approved offer. The taxonomy, the import template and the
importer follow, and a sheet that still says "Hot Deal" lands in Offers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product-import-template.xlsx
+++ b/product-import-template.xlsx
@@ -45,7 +45,7 @@
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Only for a Hot Deal: the old price, shown struck through. Leave blank otherwise.</t>
+          <t>Only for an offer: the old price, shown struck through. Leave blank otherwise.</t>
         </r>
       </text>
     </comment>
@@ -191,7 +191,7 @@
     <t>Publish</t>
   </si>
   <si>
-    <t>Hot Deal</t>
+    <t>Offers</t>
   </si>
   <si>
     <t>Hand-Tied Bouquets</t>
@@ -371,7 +371,7 @@
     <t>Prices</t>
   </si>
   <si>
-    <t>Plain numbers in Qatari riyal: 450, not 450 QAR and not 45000. Was price QAR is only for a Hot Deal — fill it in and the old price appears struck through beside the new one.</t>
+    <t>Plain numbers in Qatari riyal: 450, not 450 QAR and not 45000. Was price QAR is only for an offer — fill it in and the old price appears struck through beside the new one.</t>
   </si>
   <si>
     <t>Categories</t>

</xml_diff>